<commit_message>
Auditoría de captación y campaña de 30 días para boxes
Informe con evidencias (web, Instagram/Metricool, formulario), nicho,
oferta de entrada, guion de demo, guion comercial y seguimiento,
experimento de embudo y las 5 primeras piezas producidas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GN2RjNdyZubo7xSYMcfhZr
</commit_message>
<xml_diff>
--- a/marketing/prospeccion/prospeccion-centros-barcelona.xlsx
+++ b/marketing/prospeccion/prospeccion-centros-barcelona.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Centros" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Leyenda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centros" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leyenda" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Centros'!$A$1:$R$32</definedName>
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy hh:mm"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy hh:mm"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -92,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -100,7 +99,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -109,7 +108,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -117,6 +116,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -502,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R32"/>
+  <dimension ref="A1:T32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -523,6 +528,8 @@
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="24" customWidth="1" min="17" max="17"/>
     <col width="34" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -616,6 +623,16 @@
           <t>Notas</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Variante oferta (A/B)</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Motivo de pérdida</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -665,10 +682,10 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L2" s="3" t="n">
+      <c r="L2" s="10" t="n">
         <v>46309.92361111111</v>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="M2" s="10" t="n">
         <v>46310.44791666666</v>
       </c>
       <c r="N2" s="2">
@@ -745,8 +762,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L3" s="6" t="n"/>
-      <c r="M3" s="6" t="n"/>
+      <c r="L3" s="11" t="n"/>
+      <c r="M3" s="11" t="n"/>
       <c r="N3" s="5">
         <f>IF(AND(ISNUMBER(L3),ISNUMBER(M3)),ROUND((M3-L3)*24,1),"")</f>
         <v/>
@@ -764,6 +781,11 @@
       <c r="R3" s="5" t="inlineStr">
         <is>
           <t>Pequeña, independiente</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -813,8 +835,8 @@
           <t>Teléfono</t>
         </is>
       </c>
-      <c r="L4" s="6" t="n"/>
-      <c r="M4" s="6" t="n"/>
+      <c r="L4" s="11" t="n"/>
+      <c r="M4" s="11" t="n"/>
       <c r="N4" s="5">
         <f>IF(AND(ISNUMBER(L4),ISNUMBER(M4)),ROUND((M4-L4)*24,1),"")</f>
         <v/>
@@ -832,6 +854,11 @@
       <c r="R4" s="5" t="inlineStr">
         <is>
           <t>Pequeña; sin Instagram en la web</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -881,8 +908,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L5" s="6" t="n"/>
-      <c r="M5" s="6" t="n"/>
+      <c r="L5" s="11" t="n"/>
+      <c r="M5" s="11" t="n"/>
       <c r="N5" s="5">
         <f>IF(AND(ISNUMBER(L5),ISNUMBER(M5)),ROUND((M5-L5)*24,1),"")</f>
         <v/>
@@ -898,6 +925,11 @@
       </c>
       <c r="Q5" s="7" t="inlineStr"/>
       <c r="R5" s="5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
@@ -945,8 +977,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L6" s="6" t="n"/>
-      <c r="M6" s="6" t="n"/>
+      <c r="L6" s="11" t="n"/>
+      <c r="M6" s="11" t="n"/>
       <c r="N6" s="5">
         <f>IF(AND(ISNUMBER(L6),ISNUMBER(M6)),ROUND((M6-L6)*24,1),"")</f>
         <v/>
@@ -964,6 +996,11 @@
       <c r="R6" s="5" t="inlineStr">
         <is>
           <t>Varios centros; ya usa WhatsApp</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -1013,8 +1050,8 @@
           <t>Teléfono</t>
         </is>
       </c>
-      <c r="L7" s="6" t="n"/>
-      <c r="M7" s="6" t="n"/>
+      <c r="L7" s="11" t="n"/>
+      <c r="M7" s="11" t="n"/>
       <c r="N7" s="5">
         <f>IF(AND(ISNUMBER(L7),ISNUMBER(M7)),ROUND((M7-L7)*24,1),"")</f>
         <v/>
@@ -1032,6 +1069,11 @@
       <c r="R7" s="5" t="inlineStr">
         <is>
           <t>Datos de guia.barcelona.cat</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1069,8 +1111,8 @@
           <t>Buscar contacto</t>
         </is>
       </c>
-      <c r="L8" s="6" t="n"/>
-      <c r="M8" s="6" t="n"/>
+      <c r="L8" s="11" t="n"/>
+      <c r="M8" s="11" t="n"/>
       <c r="N8" s="5">
         <f>IF(AND(ISNUMBER(L8),ISNUMBER(M8)),ROUND((M8-L8)*24,1),"")</f>
         <v/>
@@ -1088,6 +1130,11 @@
       <c r="R8" s="5" t="inlineStr">
         <is>
           <t>Buscar Instagram/teléfono en Google Maps</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -1137,8 +1184,8 @@
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="L9" s="6" t="n"/>
-      <c r="M9" s="6" t="n"/>
+      <c r="L9" s="11" t="n"/>
+      <c r="M9" s="11" t="n"/>
       <c r="N9" s="5">
         <f>IF(AND(ISNUMBER(L9),ISNUMBER(M9)),ROUND((M9-L9)*24,1),"")</f>
         <v/>
@@ -1156,6 +1203,11 @@
       <c r="R9" s="5" t="inlineStr">
         <is>
           <t>Fuera de BCN ciudad</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1213,8 +1265,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L10" s="6" t="n"/>
-      <c r="M10" s="6" t="n"/>
+      <c r="L10" s="11" t="n"/>
+      <c r="M10" s="11" t="n"/>
       <c r="N10" s="5">
         <f>IF(AND(ISNUMBER(L10),ISNUMBER(M10)),ROUND((M10-L10)*24,1),"")</f>
         <v/>
@@ -1232,6 +1284,11 @@
       <c r="R10" s="5" t="inlineStr">
         <is>
           <t>Cadena local (~20 centros): ciclo de venta largo</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -1285,8 +1342,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L11" s="6" t="n"/>
-      <c r="M11" s="6" t="n"/>
+      <c r="L11" s="11" t="n"/>
+      <c r="M11" s="11" t="n"/>
       <c r="N11" s="5">
         <f>IF(AND(ISNUMBER(L11),ISNUMBER(M11)),ROUND((M11-L11)*24,1),"")</f>
         <v/>
@@ -1304,6 +1361,11 @@
       <c r="R11" s="5" t="inlineStr">
         <is>
           <t>Academia de barrio</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1349,8 +1411,8 @@
           <t>Teléfono</t>
         </is>
       </c>
-      <c r="L12" s="6" t="n"/>
-      <c r="M12" s="6" t="n"/>
+      <c r="L12" s="11" t="n"/>
+      <c r="M12" s="11" t="n"/>
       <c r="N12" s="5">
         <f>IF(AND(ISNUMBER(L12),ISNUMBER(M12)),ROUND((M12-L12)*24,1),"")</f>
         <v/>
@@ -1368,6 +1430,11 @@
       <c r="R12" s="5" t="inlineStr">
         <is>
           <t>+40 años; sin WhatsApp en la web</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -1421,8 +1488,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L13" s="6" t="n"/>
-      <c r="M13" s="6" t="n"/>
+      <c r="L13" s="11" t="n"/>
+      <c r="M13" s="11" t="n"/>
       <c r="N13" s="5">
         <f>IF(AND(ISNUMBER(L13),ISNUMBER(M13)),ROUND((M13-L13)*24,1),"")</f>
         <v/>
@@ -1438,6 +1505,11 @@
       </c>
       <c r="Q13" s="7" t="inlineStr"/>
       <c r="R13" s="5" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -1489,8 +1561,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L14" s="6" t="n"/>
-      <c r="M14" s="6" t="n"/>
+      <c r="L14" s="11" t="n"/>
+      <c r="M14" s="11" t="n"/>
       <c r="N14" s="5">
         <f>IF(AND(ISNUMBER(L14),ISNUMBER(M14)),ROUND((M14-L14)*24,1),"")</f>
         <v/>
@@ -1508,6 +1580,11 @@
       <c r="R14" s="5" t="inlineStr">
         <is>
           <t>4 academias en BCN</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -1557,8 +1634,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L15" s="6" t="n"/>
-      <c r="M15" s="6" t="n"/>
+      <c r="L15" s="11" t="n"/>
+      <c r="M15" s="11" t="n"/>
       <c r="N15" s="5">
         <f>IF(AND(ISNUMBER(L15),ISNUMBER(M15)),ROUND((M15-L15)*24,1),"")</f>
         <v/>
@@ -1576,6 +1653,11 @@
       <c r="R15" s="5" t="inlineStr">
         <is>
           <t>Franquicia</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1621,8 +1703,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L16" s="6" t="n"/>
-      <c r="M16" s="6" t="n"/>
+      <c r="L16" s="11" t="n"/>
+      <c r="M16" s="11" t="n"/>
       <c r="N16" s="5">
         <f>IF(AND(ISNUMBER(L16),ISNUMBER(M16)),ROUND((M16-L16)*24,1),"")</f>
         <v/>
@@ -1640,6 +1722,11 @@
       <c r="R16" s="5" t="inlineStr">
         <is>
           <t>Repaso y Selectividad</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -1689,8 +1776,8 @@
           <t>Teléfono</t>
         </is>
       </c>
-      <c r="L17" s="6" t="n"/>
-      <c r="M17" s="6" t="n"/>
+      <c r="L17" s="11" t="n"/>
+      <c r="M17" s="11" t="n"/>
       <c r="N17" s="5">
         <f>IF(AND(ISNUMBER(L17),ISNUMBER(M17)),ROUND((M17-L17)*24,1),"")</f>
         <v/>
@@ -1708,6 +1795,11 @@
       <c r="R17" s="5" t="inlineStr">
         <is>
           <t>Móvil: probable WhatsApp</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1749,8 +1841,8 @@
           <t>Teléfono</t>
         </is>
       </c>
-      <c r="L18" s="6" t="n"/>
-      <c r="M18" s="6" t="n"/>
+      <c r="L18" s="11" t="n"/>
+      <c r="M18" s="11" t="n"/>
       <c r="N18" s="5">
         <f>IF(AND(ISNUMBER(L18),ISNUMBER(M18)),ROUND((M18-L18)*24,1),"")</f>
         <v/>
@@ -1768,6 +1860,11 @@
       <c r="R18" s="5" t="inlineStr">
         <is>
           <t>Teléfono de directorio (serveisactius.cat): verificar</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -1809,8 +1906,8 @@
           <t>Buscar contacto</t>
         </is>
       </c>
-      <c r="L19" s="6" t="n"/>
-      <c r="M19" s="6" t="n"/>
+      <c r="L19" s="11" t="n"/>
+      <c r="M19" s="11" t="n"/>
       <c r="N19" s="5">
         <f>IF(AND(ISNUMBER(L19),ISNUMBER(M19)),ROUND((M19-L19)*24,1),"")</f>
         <v/>
@@ -1828,6 +1925,11 @@
       <c r="R19" s="5" t="inlineStr">
         <is>
           <t>Encontrado vía Instagram</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1869,8 +1971,8 @@
           <t>Buscar contacto</t>
         </is>
       </c>
-      <c r="L20" s="6" t="n"/>
-      <c r="M20" s="6" t="n"/>
+      <c r="L20" s="11" t="n"/>
+      <c r="M20" s="11" t="n"/>
       <c r="N20" s="5">
         <f>IF(AND(ISNUMBER(L20),ISNUMBER(M20)),ROUND((M20-L20)*24,1),"")</f>
         <v/>
@@ -1888,6 +1990,11 @@
       <c r="R20" s="5" t="inlineStr">
         <is>
           <t>Encontrado vía Instagram</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -1937,8 +2044,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L21" s="6" t="n"/>
-      <c r="M21" s="6" t="n"/>
+      <c r="L21" s="11" t="n"/>
+      <c r="M21" s="11" t="n"/>
       <c r="N21" s="5">
         <f>IF(AND(ISNUMBER(L21),ISNUMBER(M21)),ROUND((M21-L21)*24,1),"")</f>
         <v/>
@@ -1956,6 +2063,11 @@
       <c r="R21" s="5" t="inlineStr">
         <is>
           <t>Primera clase gratis</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -2009,8 +2121,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L22" s="6" t="n"/>
-      <c r="M22" s="6" t="n"/>
+      <c r="L22" s="11" t="n"/>
+      <c r="M22" s="11" t="n"/>
       <c r="N22" s="5">
         <f>IF(AND(ISNUMBER(L22),ISNUMBER(M22)),ROUND((M22-L22)*24,1),"")</f>
         <v/>
@@ -2028,6 +2140,11 @@
       <c r="R22" s="5" t="inlineStr">
         <is>
           <t>Clase de prueba gratis</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -2081,8 +2198,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L23" s="6" t="n"/>
-      <c r="M23" s="6" t="n"/>
+      <c r="L23" s="11" t="n"/>
+      <c r="M23" s="11" t="n"/>
       <c r="N23" s="5">
         <f>IF(AND(ISNUMBER(L23),ISNUMBER(M23)),ROUND((M23-L23)*24,1),"")</f>
         <v/>
@@ -2098,6 +2215,11 @@
       </c>
       <c r="Q23" s="7" t="inlineStr"/>
       <c r="R23" s="5" t="inlineStr"/>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
@@ -2141,8 +2263,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L24" s="6" t="n"/>
-      <c r="M24" s="6" t="n"/>
+      <c r="L24" s="11" t="n"/>
+      <c r="M24" s="11" t="n"/>
       <c r="N24" s="5">
         <f>IF(AND(ISNUMBER(L24),ISNUMBER(M24)),ROUND((M24-L24)*24,1),"")</f>
         <v/>
@@ -2160,6 +2282,11 @@
       <c r="R24" s="5" t="inlineStr">
         <is>
           <t>Clases de prueba gratuitas</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -2209,8 +2336,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L25" s="6" t="n"/>
-      <c r="M25" s="6" t="n"/>
+      <c r="L25" s="11" t="n"/>
+      <c r="M25" s="11" t="n"/>
       <c r="N25" s="5">
         <f>IF(AND(ISNUMBER(L25),ISNUMBER(M25)),ROUND((M25-L25)*24,1),"")</f>
         <v/>
@@ -2228,6 +2355,11 @@
       <c r="R25" s="5" t="inlineStr">
         <is>
           <t>Clase gratis</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -2281,8 +2413,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L26" s="6" t="n"/>
-      <c r="M26" s="6" t="n"/>
+      <c r="L26" s="11" t="n"/>
+      <c r="M26" s="11" t="n"/>
       <c r="N26" s="5">
         <f>IF(AND(ISNUMBER(L26),ISNUMBER(M26)),ROUND((M26-L26)*24,1),"")</f>
         <v/>
@@ -2298,6 +2430,11 @@
       </c>
       <c r="Q26" s="7" t="inlineStr"/>
       <c r="R26" s="5" t="inlineStr"/>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
@@ -2349,8 +2486,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L27" s="6" t="n"/>
-      <c r="M27" s="6" t="n"/>
+      <c r="L27" s="11" t="n"/>
+      <c r="M27" s="11" t="n"/>
       <c r="N27" s="5">
         <f>IF(AND(ISNUMBER(L27),ISNUMBER(M27)),ROUND((M27-L27)*24,1),"")</f>
         <v/>
@@ -2366,6 +2503,11 @@
       </c>
       <c r="Q27" s="7" t="inlineStr"/>
       <c r="R27" s="5" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
@@ -2409,8 +2551,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L28" s="6" t="n"/>
-      <c r="M28" s="6" t="n"/>
+      <c r="L28" s="11" t="n"/>
+      <c r="M28" s="11" t="n"/>
       <c r="N28" s="5">
         <f>IF(AND(ISNUMBER(L28),ISNUMBER(M28)),ROUND((M28-L28)*24,1),"")</f>
         <v/>
@@ -2426,6 +2568,11 @@
       </c>
       <c r="Q28" s="7" t="inlineStr"/>
       <c r="R28" s="5" t="inlineStr"/>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
@@ -2469,8 +2616,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L29" s="6" t="n"/>
-      <c r="M29" s="6" t="n"/>
+      <c r="L29" s="11" t="n"/>
+      <c r="M29" s="11" t="n"/>
       <c r="N29" s="5">
         <f>IF(AND(ISNUMBER(L29),ISNUMBER(M29)),ROUND((M29-L29)*24,1),"")</f>
         <v/>
@@ -2488,6 +2635,11 @@
       <c r="R29" s="5" t="inlineStr">
         <is>
           <t>Ya usa un CRM (GoHighLevel)</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -2537,8 +2689,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L30" s="6" t="n"/>
-      <c r="M30" s="6" t="n"/>
+      <c r="L30" s="11" t="n"/>
+      <c r="M30" s="11" t="n"/>
       <c r="N30" s="5">
         <f>IF(AND(ISNUMBER(L30),ISNUMBER(M30)),ROUND((M30-L30)*24,1),"")</f>
         <v/>
@@ -2556,6 +2708,11 @@
       <c r="R30" s="5" t="inlineStr">
         <is>
           <t>Reservas por WhatsApp</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -2609,8 +2766,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L31" s="6" t="n"/>
-      <c r="M31" s="6" t="n"/>
+      <c r="L31" s="11" t="n"/>
+      <c r="M31" s="11" t="n"/>
       <c r="N31" s="5">
         <f>IF(AND(ISNUMBER(L31),ISNUMBER(M31)),ROUND((M31-L31)*24,1),"")</f>
         <v/>
@@ -2628,6 +2785,11 @@
       <c r="R31" s="5" t="inlineStr">
         <is>
           <t>Reservas por WhatsApp; 3 estudios</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -2673,8 +2835,8 @@
           <t>Instagram DM</t>
         </is>
       </c>
-      <c r="L32" s="6" t="n"/>
-      <c r="M32" s="6" t="n"/>
+      <c r="L32" s="11" t="n"/>
+      <c r="M32" s="11" t="n"/>
       <c r="N32" s="5">
         <f>IF(AND(ISNUMBER(L32),ISNUMBER(M32)),ROUND((M32-L32)*24,1),"")</f>
         <v/>
@@ -2690,15 +2852,26 @@
       </c>
       <c r="Q32" s="7" t="inlineStr"/>
       <c r="R32" s="5" t="inlineStr"/>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:R32"/>
-  <dataValidations count="2">
-    <dataValidation sqref="P2:P32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Pendiente,Prueba hecha,Contactado,Respondió,Llamada agendada,Cliente,No interesado"</formula1>
+  <dataValidations count="4">
+    <dataValidation sqref="P2:P200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pendiente,Prueba hecha,Contactado,Respondió,Demo hecha,Propuesta,Cliente,No interesado"</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Alta,Media,Baja"</formula1>
+    </dataValidation>
+    <dataValidation sqref="S2:S200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"A,B"</formula1>
+    </dataValidation>
+    <dataValidation sqref="T2:T200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No responde,No ve el problema,Precio,Tiempo/montaje,Confianza (sois nuevos),Otro"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2712,7 +2885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2794,6 +2967,27 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Experimento (campaña boxes, ver marketing/campana-boxes/INFORME.md §8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Columna S: variante de oferta. Impares = A (precios web 590 € + 89 €/mes), pares = B (piloto 149 € con garantía).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Columna T: motivo de pérdida, una sola opción. Rellenarla siempre que un centro se caiga del embudo.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>